<commit_message>
Gap-fill Wave 2 Financial: 44 verified (24 Yes / 10 Stretch / 10 No)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TE8a9ptd2NGPUtY6iZfzkb
</commit_message>
<xml_diff>
--- a/reports/F1-Master-Mirror-GapFill-2026-09.xlsx
+++ b/reports/F1-Master-Mirror-GapFill-2026-09.xlsx
@@ -15,6 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travel &amp; Hospitality" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Media &amp; Gaming" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REJECTS - No" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Banking &amp; Insurance" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trading &amp; Crypto" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -98,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -134,6 +136,21 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -500,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -531,6 +548,190 @@
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Waves 2-12 pending: Financial -&gt; Health -&gt; Tech hardware -&gt; Software -&gt; Industrial -&gt; Energy -&gt; Services -&gt; Telecom/Space -&gt; Logistics/Mobility -&gt; Media/Gaming -&gt; AI. Feeds already collected: finance 49, health 53, industrial 47, tech 30, services 50, energy 46.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Wave 2 - Financial (20 Sep 2026): 44 verified -&gt; 24 Yes / 10 Stretch / 10 No. Key catches: Grupo Inbursa (Slim/Escuderia Telmex-Perez-Cadillac conflict), Topdanmark (Sampo-absorbed), Banca Generali (live MPS takeover), Brighthouse (take-private), Coinbase (roster). Asian/LATAM financials much larger than estimated (Orix $43B, Credicorp $30B).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="48" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>hq</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>ownership</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>sells (what &amp; to whom)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>headcount_band</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>revenue (date, source)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>valuation (date)</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>fit 0-4</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>fit detail</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>soft flags</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>verdict reason</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>best angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Yuanta Financial Holdings</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>Public (TWSE); Ho family influence, broad institutional ownership; no state ownership found</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Securities brokerage, banking, insurance, asset management, with a regional ETF franchise (Yuanta ETFs) distributed across Taiwan, and other Asian markets</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>10k-25k (~16,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>TTM revenue ~$4.13B USD (Aug 2026), up from ~$3.75B in 2024 - growing</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>Market cap ~$28.0B USD as of July 2026 (NT$967.7B) - well above input's ~$9B estimate; verified current</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L2" s="7" t="inlineStr">
+        <is>
+          <t>Regional ETF/brokerage franchise sells across 3+ Asian markets - pass; investor/trader client base skews affluent, decision-making individuals - pass; brokerage/trading naturally supports a speed-precision-data performance story that maps well to F1 - pass; category open - no major Asian broker/exchange on the F1 grid (brokers/exchanges are the Trading &amp; Crypto bucket, largely untapped). Investor/trader customer scale (pass, note). No F1/motorsport sponsorship found.</t>
+        </is>
+      </c>
+      <c r="M2" s="7" t="inlineStr"/>
+      <c r="N2" s="7" t="inlineStr">
+        <is>
+          <t>Mega-cap regional broker/ETF platform with a strong trading-performance narrative, multi-market reach, and no existing F1 tie</t>
+        </is>
+      </c>
+      <c r="O2" s="7" t="inlineStr">
+        <is>
+          <t>"Precision execution, real-time performance" trading narrative tied to F1 speed/data themes, targeting affluent retail and institutional investors across Yuanta's multi-market ETF/brokerage footprint</t>
         </is>
       </c>
     </row>
@@ -5923,7 +6124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7683,6 +7884,3237 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>AMMB Holdings (AmBank Group)</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>Public (Bursa Malaysia); ANZ fully exited (last 5.17% sold June 2024) - no single disclosed controlling shareholder, dispersed institutional ownership; no state control found</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>Banking, insurance, investment banking to Malaysian consumers/corporates</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>&lt;10k (~8,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>TTM revenue ~$1.28-1.3B USD (Sept 2026) - roughly matches input's ~$1B estimate, modest growth</t>
+        </is>
+      </c>
+      <c r="J25" s="13" t="inlineStr">
+        <is>
+          <t>Market cap ~$5.55-5.7B USD as of Sept 2026 - above input's ~$3.5B "borderline" estimate, so the market-cap concern is resolved, but still well below the $10B mega-brand bar and the smallest cap in this batch</t>
+        </is>
+      </c>
+      <c r="K25" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>Single-market Malaysia-only bank - fails 3+ market test; mass retail/business banking buyers, not a distinctly affluent segment; no performance-tech-precision story; category technically open but weak overall narrative given scale. Mass-market customer scale (pass, note). No F1/motorsport sponsorship found.</t>
+        </is>
+      </c>
+      <c r="M25" s="13" t="inlineStr">
+        <is>
+          <t>Legacy 1MDB corruption scandal - AmBank paid RM2.83B settlement to the Malaysian government (2021); fully settled and cash received, but the historic governance/reputational overhang is worth a compliance check before outreach</t>
+        </is>
+      </c>
+      <c r="N25" s="13" t="inlineStr">
+        <is>
+          <t>Sub-scale (well below mega-brand threshold), single-market bank with legacy 1MDB governance history and a weak affluent-brand narrative</t>
+        </is>
+      </c>
+      <c r="O25" s="13" t="inlineStr">
+        <is>
+          <t>Not recommended this wave; if revisited, would need to lead with post-1MDB governance turnaround credibility rather than a premium-brand story</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>IndusInd Bank</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>Public (NSE/BSE); Hinduja Group promoter-controlled, private - no state ownership</t>
+        </is>
+      </c>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>Retail and corporate banking, vehicle finance to Indian consumers/businesses</t>
+        </is>
+      </c>
+      <c r="H26" s="14" t="inlineStr">
+        <is>
+          <t>25k-50k (~40,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>Input's ~$4B FY2024 estimate stands unverified this pass (est.) - not independently re-confirmed</t>
+        </is>
+      </c>
+      <c r="J26" s="13" t="inlineStr">
+        <is>
+          <t>Market cap ~₹73,746 Cr (~US$8.4B at ~88 INR/USD) as of Sept 17, 2026 - stock up 33.6% over the last year, recovering but still below the pre-crisis $10B+ level noted in input; verified current (currency-converted)</t>
+        </is>
+      </c>
+      <c r="K26" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t>Single-market India-only bank - fails 3+ market test; mass retail/vehicle-finance buyers, not distinctly affluent; category technically open but capacity concern dominates. Mass-market customer scale (pass, note). No F1/motorsport sponsorship found.</t>
+        </is>
+      </c>
+      <c r="M26" s="13" t="inlineStr">
+        <is>
+          <t>2025 derivatives/accounting lapse triggered a CEO exit and governance scrutiny (per input) - capacity/marketing appetite likely still constrained; stock has since recovered (+33.6% YoY, active investor-relations outreach Sept 2026) suggesting an improving but still fresh situation</t>
+        </is>
+      </c>
+      <c r="N26" s="13" t="inlineStr">
+        <is>
+          <t>Still working through a 2025 governance/accounting crisis - capacity and sponsorship appetite too fresh/impaired to prioritize this wave despite share-price recovery</t>
+        </is>
+      </c>
+      <c r="O26" s="13" t="inlineStr">
+        <is>
+          <t>Revisit in a future wave once the post-crisis leadership and governance reset is further along</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Grupo Financiero Inbursa</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>Mexico City, Mexico</t>
+        </is>
+      </c>
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>Controlled by Carlos Slim and family (majority private ownership); listed on BMV. No state or sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="G27" s="13" t="inlineStr">
+        <is>
+          <t>Banking, insurance, brokerage, and pensions to Mexican consumers and corporates</t>
+        </is>
+      </c>
+      <c r="H27" s="14" t="inlineStr">
+        <is>
+          <t>~15,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>~$2.5B annualized run-rate, 2026 (Q2 2026 revenue 11.8B MXN, down 14% YoY) - Inbursa 1Q26/investing.com</t>
+        </is>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>~$15.0B market cap as of Sep 2026 (260.4B MXN) - companiesmarketcap</t>
+        </is>
+      </c>
+      <c r="K27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="13" t="inlineStr">
+        <is>
+          <t>Financially it would exceed the bar (mega-cap, well above thresholds), but Inbursa fails the F1-exposure screen: its controlling shareholder, Carlos Slim, personally founded and funds Escuderia Telmex, the motorsport program that has backed Sergio Perez's F1 career for over 20 years - including his newly confirmed, multi-year 2026 return with the Cadillac F1 team. This is an active, current, high-profile parent/family F1 tie (via Telmex/America Movil, both Slim-controlled), directly conflicting with a fresh sponsorship pitch to the same family's financial arm.</t>
+        </is>
+      </c>
+      <c r="M27" s="13" t="inlineStr">
+        <is>
+          <t>Revenue and net income declining YoY through 2026 (Q2 2026 net income down 28% YoY) - separate concern even setting aside F1 conflict</t>
+        </is>
+      </c>
+      <c r="N27" s="13" t="inlineStr">
+        <is>
+          <t>Parent/family F1 tie: Carlos Slim's Escuderia Telmex actively sponsors Sergio Perez at Cadillac F1 for the 2026 season - direct conflict of interest.</t>
+        </is>
+      </c>
+      <c r="O27" s="13" t="inlineStr">
+        <is>
+          <t>N/A - deprioritize; the Slim family's F1 relationship runs through Telmex/America Movil, not Inbursa, so any future F1 commercial conversation with this ownership group should go through the existing Escuderia Telmex relationship rather than as a new sponsor pitch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Topdanmark</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Ballerup, Denmark</t>
+        </is>
+      </c>
+      <c r="F28" s="14" t="inlineStr">
+        <is>
+          <t>~92.6% owned by Sampo Group (Finland); DELISTED from Nasdaq Copenhagen in 2024 following Sampo's exchange offer</t>
+        </is>
+      </c>
+      <c r="G28" s="13" t="inlineStr">
+        <is>
+          <t>P&amp;C and life insurance in Denmark</t>
+        </is>
+      </c>
+      <c r="H28" s="14" t="inlineStr">
+        <is>
+          <t>~2,500 (est.)</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="inlineStr">
+        <is>
+          <t>~$1.8B (est., FY2024 pre-delisting; no longer independently reported post-Sampo integration)</t>
+        </is>
+      </c>
+      <c r="J28" s="13" t="inlineStr">
+        <is>
+          <t>Delisted 2024; last implied deal value ~$4.7B in Sampo's 2024 exchange offer (source: Yahoo Finance/Sampo.com)</t>
+        </is>
+      </c>
+      <c r="K28" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>Financially sound but no longer an independent decision-making entity - Sampo Group (Helsinki) holds ~92.6% and delisted the stock in 2024, so sponsorship/marketing budget authority sits with the parent, not Topdanmark.</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="inlineStr">
+        <is>
+          <t>Input mischaracterized Sampo's position as a 'minority strategic investor' - it is now a ~92.6% controlling parent post-delisting; Company no longer independently listed/reported</t>
+        </is>
+      </c>
+      <c r="N28" s="13" t="inlineStr">
+        <is>
+          <t>Fails the capacity/independence test: majority-owned (92.6%) and delisted by parent Sampo Group in 2024, so Topdanmark itself cannot be the sponsorship decision-maker.</t>
+        </is>
+      </c>
+      <c r="O28" s="13" t="inlineStr">
+        <is>
+          <t>Not viable as a standalone target; any interest should be redirected to Sampo Group as the controlling entity (separate lead, not this one).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>Banca Generali</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Trieste/Milan, Italy</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Assicurazioni Generali holds 50.17% (majority parent); as of Aug 2026 Banca Generali is also the target of an irrevocable, live all-share takeover bid from Monte dei Paschi (MPS) valuing it at ~EUR 8.7B, part of a wider Italian banking consolidation battle (Intesa Sanpaolo vs MPS vs Banco BPM)</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>Wealth management and private banking to Italian affluent clients</t>
+        </is>
+      </c>
+      <c r="H29" s="14" t="inlineStr">
+        <is>
+          <t>~1,700 (est.)</t>
+        </is>
+      </c>
+      <c r="I29" s="13" t="inlineStr">
+        <is>
+          <t>~€992-999M FY2024/FY2025 (source: stockanalysis.com)</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>€6.85B market cap as of 11 Jun 2026 (source: companiesmarketcap.com); MPS bid values it at ~€8.7B</t>
+        </is>
+      </c>
+      <c r="K29" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" s="13" t="inlineStr">
+        <is>
+          <t>Growing wealth manager with a strong Italian F1 fan-base angle (Monza), but currently mid-way through a live, irrevocable MPS takeover offer (acceptance period expected Dec 2026-Feb 2027) layered on top of majority ownership by Assicurazioni Generali - a textbook 'major restructuring in progress' disqualifier right now.</t>
+        </is>
+      </c>
+      <c r="M29" s="13" t="inlineStr">
+        <is>
+          <t>Live MPS takeover bid announced 21 Aug 2026, irrevocable even amid a separate Intesa Sanpaolo hostile bid for MPS itself - ownership/strategy in flux into 2027; Majority-owned (50.17%) by Assicurazioni Generali, which is already captured separately in the sponsorship database per input flag</t>
+        </is>
+      </c>
+      <c r="N29" s="13" t="inlineStr">
+        <is>
+          <t>Fails the 'no major restructuring' capacity test - subject to a live, irrevocable takeover bid and broader Italian bank-consolidation fight as of Sept 2026, with resolution not expected before 2027; also majority-controlled by an already-captured parent (Generali).</t>
+        </is>
+      </c>
+      <c r="O29" s="13" t="inlineStr">
+        <is>
+          <t>Not viable now - revisit post-resolution of the MPS/BPM/Intesa consolidation (est. mid-2027 earliest).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Investor AB</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Stockholm, Sweden</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Controlled by the Knut and Alice Wallenberg Foundation (20.07% of capital, 42.96% of votes) - foundation/family-controlled, not state or sovereign</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="inlineStr">
+        <is>
+          <t>Investment holding company with stakes in Atlas Copco, Ericsson, ABB, AstraZeneca, EQT, etc.</t>
+        </is>
+      </c>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t>~300 (est., holding-company level only)</t>
+        </is>
+      </c>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>Not applicable - NAV/dividend-based holding company</t>
+        </is>
+      </c>
+      <c r="J30" s="13" t="inlineStr">
+        <is>
+          <t>SEK 1.24 trillion market cap as of 18 Sept 2026 (~$118B), +43% YoY (source: tradingeconomics.com)</t>
+        </is>
+      </c>
+      <c r="K30" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" s="13" t="inlineStr">
+        <is>
+          <t>Enormous market cap but a pure investment holding vehicle with no products, customers, or marketing function of its own. Checked for portfolio-company F1 exposure (e.g., Ericsson) - found none; the only 'Ericsson' link in F1 is unrelated driver Marcus Ericsson.</t>
+        </is>
+      </c>
+      <c r="M30" s="13" t="inlineStr">
+        <is>
+          <t>Foundation-controlled decision-making (Wallenberg) concentrates authority outside a normal marketing/sponsorship function; No consumer-facing brand or customer base to activate via F1</t>
+        </is>
+      </c>
+      <c r="N30" s="13" t="inlineStr">
+        <is>
+          <t>Despite mega-cap scale, Investor AB has no customer base or brand proposition for F1 to serve - it is a passive holding company, not an operating consumer or B2B brand.</t>
+        </is>
+      </c>
+      <c r="O30" s="13" t="inlineStr">
+        <is>
+          <t>Not viable as the holding company; if there is interest, it should be evaluated portfolio-company by portfolio-company (e.g., Atlas Copco, ABB) rather than at the parent level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>Coinbase Global, Inc.</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>Remote-first / San Francisco/New York, USA</t>
+        </is>
+      </c>
+      <c r="F31" s="14" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: COIN); Brian Armstrong holds super-voting Class B shares but no state/sovereign ownership</t>
+        </is>
+      </c>
+      <c r="G31" s="13" t="inlineStr">
+        <is>
+          <t>Cryptocurrency exchange and custody services for retail and institutional clients globally</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>3,000–5,000</t>
+        </is>
+      </c>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>~$7.2B FY2025 total revenue (net revenue ~$6.9B), up 9% YoY, per FY2025 shareholder letter/10-K</t>
+        </is>
+      </c>
+      <c r="J31" s="13" t="inlineStr">
+        <is>
+          <t>~$49–50B market cap as of mid-Sept 2026 (MacroTrends)</t>
+        </is>
+      </c>
+      <c r="K31" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="L31" s="13" t="inlineStr">
+        <is>
+          <t>Largest US crypto exchange, profitable in 2025, doubled trading volume/market share, no restructuring. Huge global retail+institutional customer base. F1 exposure: category is crowded — Crypto.com holds official F1 global partner/naming-rights status (Miami GP) and other crypto brands (Bybit–McLaren, historically Tezos–Red Bull, OKX–McLaren) already occupy team-level slots; Coinbase itself has no existing F1 deal. No sovereign ownership issue.</t>
+        </is>
+      </c>
+      <c r="M31" s="13" t="inlineStr">
+        <is>
+          <t>Series-level (F1 global partner) category likely blocked by Crypto.com's existing exclusivity — check exclusivity clauses before pitching at that tier; Crypto-price volatility affects marketing-budget stability year to year</t>
+        </is>
+      </c>
+      <c r="N31" s="13" t="inlineStr">
+        <is>
+          <t>F1 sponsor roster conflict (confirmed in prior audit) - excluded regardless of category logic.</t>
+        </is>
+      </c>
+      <c r="O31" s="13" t="inlineStr">
+        <is>
+          <t>Target a specific team without an existing crypto sponsor for a team-level (not series-level) partnership, leaning on Coinbase's institutional/custody credibility rather than pure retail-trading hype.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>Brighthouse Financial, Inc.</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Charlotte, NC, USA</t>
+        </is>
+      </c>
+      <c r="F32" s="14" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: BHF) but under a signed, stockholder-approved merger agreement to be acquired by Aquarian Capital LLC for ~$4.1B ($70/share cash); HSR cleared, awaiting insurance-regulator approvals, expected to close in 2026</t>
+        </is>
+      </c>
+      <c r="G32" s="13" t="inlineStr">
+        <is>
+          <t>Annuities and life insurance for US consumers</t>
+        </is>
+      </c>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>1,000–2,000</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>$6.77B FY2025 (up sharply from $4.72B FY2024, driven largely by reinsurance/actuarial items rather than core organic growth), per Q4/FY2025 results</t>
+        </is>
+      </c>
+      <c r="J32" s="13" t="inlineStr">
+        <is>
+          <t>~$3.4B market cap as of 11 Aug 2026 (consistent with the pending $4.1B enterprise-value buyout)</t>
+        </is>
+      </c>
+      <c r="K32" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" s="13" t="inlineStr">
+        <is>
+          <t>Financially the FY2025 top line looks strong, but the take-private deal (announced Nov 2025, stockholders approved Feb 2026) is the dominant fact: the company is mid-transaction with an as-yet-uncertain post-close ownership posture (Aquarian Capital, a PE-backed insurance holding company) and marketing/sponsorship decision-making authority in flux. No F1 exposure otherwise. No sovereign ownership, but effectively a moving target.</t>
+        </is>
+      </c>
+      <c r="M32" s="13" t="inlineStr">
+        <is>
+          <t>Pending acquisition by Aquarian Capital — deal not yet closed as of the most recent public data (still pending insurance regulatory approval as of mid-2026); verify closing status immediately before any outreach; Q4 2025 profit was described as weak despite full-year revenue growth — earnings quality mixed</t>
+        </is>
+      </c>
+      <c r="N32" s="13" t="inlineStr">
+        <is>
+          <t>Company is in the final stages of a $4.1B take-private acquisition by Aquarian Capital; committing sponsorship outreach to a target mid-ownership-change is premature until the deal closes and new capital-allocation priorities are known.</t>
+        </is>
+      </c>
+      <c r="O32" s="13" t="inlineStr">
+        <is>
+          <t>Revisit post-close under Aquarian Capital ownership once the acquisition is finalized and new management's marketing posture is clear — not viable as a Wave 2 target today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>Genworth Financial, Inc.</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>Richmond, VA, USA</t>
+        </is>
+      </c>
+      <c r="F33" s="14" t="inlineStr">
+        <is>
+          <t>Public (NYSE: GNW); majority owner of Enact Holdings (mortgage insurance); no sovereign/state stake</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>Long-term care and mortgage insurance (via majority-owned Enact Holdings) for US consumers and lenders</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
+          <t>2,000–3,000</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>$7.30B FY2025 consolidated total revenues (premiums $3.50B, net investment income $3.13B, other), per FY2025 10-K</t>
+        </is>
+      </c>
+      <c r="J33" s="13" t="inlineStr">
+        <is>
+          <t>~$3.8B market cap as of 18 Sept 2026 (above the input's flagged $3B threshold, confirmed current)</t>
+        </is>
+      </c>
+      <c r="K33" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" s="13" t="inlineStr">
+        <is>
+          <t>Honest capital-position check: consolidated legacy-insurance RBC ratio was ~289% at Q1 2026, down from ~300% at YE2025 due to a statutory loss — still above typical regulatory-comfort thresholds but moving the wrong direction quarter over quarter. More importantly, holding-company (Genworth Holdings) unrestricted cash was only ~$166M at Q1 2026 — thin liquidity for a company considering a large, multi-year global sponsorship commitment. The long-term-care turnaround (cumulative ~$34.5B NPV of approved rate increases since 2012) is real progress but the block remains a structural legacy overhang. No F1 exposure.</t>
+        </is>
+      </c>
+      <c r="M33" s="13" t="inlineStr">
+        <is>
+          <t>Holdco liquidity is thin (~$166M unrestricted cash) relative to a marquee sponsorship-scale commitment; RBC ratio declined QoQ (300%→289%) — confirm trend has stabilized before any outreach; Market cap sits close to the large-cap screening threshold — re-verify at time of outreach</t>
+        </is>
+      </c>
+      <c r="N33" s="13" t="inlineStr">
+        <is>
+          <t>Capital position is 'improving' in the sense of a multi-year LTC turnaround story, but holding-company liquidity is thin and the RBC trend ticked down last quarter — this is not a company with clear uncommitted capacity for a large discretionary sponsorship right now.</t>
+        </is>
+      </c>
+      <c r="O33" s="13" t="inlineStr">
+        <is>
+          <t>Not recommended for this wave; if capital position stabilizes and holdco liquidity rebuilds, a future long-term-care-awareness/financial-wellness angle could be revisited.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>Goosehead Insurance, Inc.</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>Westlake, TX, USA</t>
+        </is>
+      </c>
+      <c r="F34" s="14" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: GSHD); founder Mark Miller retains a large stake — no sovereign/state ownership</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>Independent insurance agency/franchise distribution platform for US homeowners and auto insurance buyers</t>
+        </is>
+      </c>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t>2,000–3,000 (mostly corporate + franchise sales agents; franchisees are independent)</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="inlineStr">
+        <is>
+          <t>~$365.3M FY2025 total revenue (up 16% YoY: Q1 $75.6M, Q2 $94.0M, Q3 $90.4M, Q4 $105.3M), per Q4/FY2025 results</t>
+        </is>
+      </c>
+      <c r="J34" s="13" t="inlineStr">
+        <is>
+          <t>~$2.43B market cap as of 3 Sept 2026, down 22% over the prior year</t>
+        </is>
+      </c>
+      <c r="K34" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" s="13" t="inlineStr">
+        <is>
+          <t>Growing revenue (+16%) but a shrinking market cap (-22% YoY) points to growth-stock/valuation volatility rather than a stable large-cap marketing budget. At ~$365M in annual revenue, a meaningful F1 sponsorship commitment (typically tens of millions annually) would represent a disproportionate share of revenue for a company this size — this is really a mid-cap growth insurtech, not a true large-cap. No F1 exposure. No ownership concerns.</t>
+        </is>
+      </c>
+      <c r="M34" s="13" t="inlineStr">
+        <is>
+          <t>Revenue small relative to market cap and relative to typical F1 sponsorship cost — confirm actual discretionary marketing budget before any pitch; Market cap down 22% YoY — check for franchise-agent attrition or other headwinds behind the decline</t>
+        </is>
+      </c>
+      <c r="N34" s="13" t="inlineStr">
+        <is>
+          <t>Revenue scale (~$365M) is too small to plausibly support a global F1-tier sponsorship, and the declining market cap suggests this is not the moment for a large discretionary marketing commitment.</t>
+        </is>
+      </c>
+      <c r="O34" s="13" t="inlineStr">
+        <is>
+          <t>Not a fit for a marquee F1 deal; if pursued at all, would only work as a very small, local/team-level activation tied to homeowner/auto-insurance messaging.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="48" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>tier</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>hq</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>ownership</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>sells (what &amp; to whom)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>headcount_band</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>revenue (date, source)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>valuation (date)</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>fit 0-4</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>fit detail</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>soft flags</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>verdict reason</t>
+        </is>
+      </c>
+      <c r="O1" s="4" t="inlineStr">
+        <is>
+          <t>best angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Aditya Birla Capital</t>
+        </is>
+      </c>
+      <c r="E2" s="15" t="inlineStr">
+        <is>
+          <t>Mumbai, India</t>
+        </is>
+      </c>
+      <c r="F2" s="15" t="inlineStr">
+        <is>
+          <t>Aditya Birla Group (Kumar Mangalam Birla family, majority promoter control) with public float on NSE/BSE. No state or sovereign ownership. (Distinct from Aditya Birla Insulators - separate group entity, confirmed no naming overlap.)</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>NBFC lending, life/health insurance, and asset management under the Aditya Birla Group umbrella</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>~30,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I2" s="7" t="inlineStr">
+        <is>
+          <t>$6.12B consolidated revenue, FY2026 (ended Mar-2026: Rs 53,871 Cr, +14% YoY) - Eulerpool/company results</t>
+        </is>
+      </c>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>~$12.6B market cap as of early Aug 2026 (~Rs 1.11 lakh Cr; +70% YoY, crossed Rs 1 lakh Cr milestone in 2026) - multibagg/stockanalysis</t>
+        </is>
+      </c>
+      <c r="K2" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2" s="7" t="inlineStr">
+        <is>
+          <t>Substantially exceeds prior estimates (market cap +58% and revenue +53% vs the Wave input's rough figures). Strong, improving profitability (Q4 FY26 consol. PAT +30% YoY) with no restructuring. Part of the globally recognized Aditya Birla Group (cement, metals, fashion, telecom with international manufacturing footprint), giving it real mega-brand marketing reach and budget appetite. No F1/motorsport tie found for Aditya Birla Capital or the parent group.</t>
+        </is>
+      </c>
+      <c r="M2" s="7" t="inlineStr">
+        <is>
+          <t>Ensure outreach is clearly targeted at Aditya Birla Capital (financial services arm) and not confused with other Birla Group listed entities</t>
+        </is>
+      </c>
+      <c r="N2" s="7" t="inlineStr">
+        <is>
+          <t>Mega-brand-scale, fast-growing, highly profitable financial arm of a globally known conglomerate with a clean F1/ownership profile.</t>
+        </is>
+      </c>
+      <c r="O2" s="7" t="inlineStr">
+        <is>
+          <t>Leverage Aditya Birla Group's existing global industrial/manufacturing footprint and brand-investment appetite; growth-stage financial-services story fits F1's push into emerging high-growth markets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C3" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
+          <t>Credicorp</t>
+        </is>
+      </c>
+      <c r="E3" s="15" t="inlineStr">
+        <is>
+          <t>Lima, Peru (Bermuda-incorporated holding company)</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>Widely held with significant long-standing family/institutional shareholders (incl. Romero family interests); NYSE-listed (BAP), no single controlling shareholder, no state or sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Banking (BCP), insurance (Pacifico), pensions (Prima AFP), and microfinance across Peru and the Andean region</t>
+        </is>
+      </c>
+      <c r="H3" s="15" t="inlineStr">
+        <is>
+          <t>~35,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>~$7.6-8.2B TTM revenue (Q2 2026 quarterly $2.17B; FY2025 annual $7.62B, +8.9% YoY) - stockanalysis/macrotrends</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>$30.3B market cap as of 12 Sep 2026 (79.4M shares) - Morningstar/stockanalysis</t>
+        </is>
+      </c>
+      <c r="K3" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>Market cap nearly double the Wave input's $16B estimate - Credicorp is a genuine regional mega-brand, NYSE-listed, dominant across Peru/Andean banking, insurance and pensions. Highly profitable and stable, no restructuring. Large, diversified customer base (retail, corporate, microfinance). Searched specifically for BCP/Credicorp/Interbank motorsport ties - none found.</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr"/>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>Largest, most profitable name in this batch with clean ownership and no F1 conflicts.</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>Flagship regional-champion pitch: dominant Andean financial brand with NYSE visibility and marketing budget scale to match a top-tier F1 partnership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Swiss Life Holding</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Zurich, Switzerland</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>Publicly listed (SIX: SLHN), widely held free float, no state/founder majority stake identified</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Life insurance, pensions, and asset management across Switzerland, France, Germany and broader Europe</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>~11,000 (est.) core group employees</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>CHF 11.7B FY2025 (~$13.2B); company guiding CHF 12.8B for 2026 (source: Simply Wall St / companiesmarketcap.com, Aug 2026)</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>CHF 26.7B market cap as of 13 Aug 2026 (~$30B) (source: ad-hoc-news.de)</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Blue-chip Swiss insurer (SMI constituent), net income and EPS both up YoY in FY2025, no restructuring underway, no state/sovereign ownership, no identified F1/motorsport sponsorship conflict for the company or any parent.</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="inlineStr">
+        <is>
+          <t>Headcount is an estimate (public disclosures cite 10,700-12,000 depending on scope); FY2025 top-line dipped 2.3% before a guided rebound - watch for confirmation in FY2026 results</t>
+        </is>
+      </c>
+      <c r="N4" s="7" t="inlineStr">
+        <is>
+          <t>Large, profitable, growing mega-cap insurer with no ownership or restructuring red flags and no competing F1 tie to clear.</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="inlineStr">
+        <is>
+          <t>Pan-European retail insurance/pensions brand looking for premium visibility - tie into F1's European calendar (Monaco, Spa, Monza) and wealth/pension-planning hospitality activations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C5" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D5" s="15" t="inlineStr">
+        <is>
+          <t>ASR Nederland (a.s.r.)</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>Utrecht, Netherlands</t>
+        </is>
+      </c>
+      <c r="F5" s="15" t="inlineStr">
+        <is>
+          <t>Fully privatized; Dutch State (via NLFI) completed full divestment of its stake in September 2017 - no residual state ownership</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Life, non-life insurance and pensions in the Netherlands</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>~5,000 (est.; likely higher post-Aegon Netherlands merger)</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>€21.2B FY2025 gross (premiums + investment income) (source: alphaspread.com/ad-hoc-news.de)</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>~€14.4B / ~$16B market cap as of Sept 2026 (source: companiesmarketcap.com/stockanalysis.com)</t>
+        </is>
+      </c>
+      <c r="K5" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Now the largest Dutch insurer post-Aegon Netherlands merger, fully state-divested since 2017 (cleaner than the input's '2023' estimate), profitable with rising 2025 profit picture, no F1 conflict found.</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr"/>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>Mega-cap, fully private, profitable and growing post-merger insurer with no ownership or capacity red flags.</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>Post-merger 'largest Dutch insurer' growth story, with a natural home-market tie-in to the Dutch Grand Prix at Zandvoort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Aflac Incorporated</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Columbus, GA, USA</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>Public (NYSE: AFL); widely held, no controlling shareholder</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Supplemental health and life insurance in the US and Japan</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>10,000–20,000</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>$17.2B FY2025 total revenues (down 9.3% from $18.9B FY2024, mainly yen/hedging-driven, not fundamental), per Q4 2025 earnings release</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>~$57–60B market cap (Sept 2026; stock ~$117/share early Sept 2026, off all-time high $128.90 in Jul 2026)</t>
+        </is>
+      </c>
+      <c r="K6" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" s="7" t="inlineStr">
+        <is>
+          <t>Highly profitable (Q4 2025 net earnings $1.4B alone), strong capital, no restructuring. Massive dual US/Japan consumer base and an iconic, globally recognizable mascot (the Aflac Duck). No F1 or motorsport exposure/conflicts found; long history of major US sports sponsorship (MLB, college football) shows real sponsorship budget and appetite. Fully public, no sovereign/parent ownership issue.</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>Revenue decline YoY is FX/hedging-driven — confirm this doesn't signal a pullback in discretionary marketing spend; Check spelling/brand variants (Aflac vs. AFLAC) in outreach materials</t>
+        </is>
+      </c>
+      <c r="N6" s="7" t="inlineStr">
+        <is>
+          <t>Mega-cap, mascot-led global consumer brand with proven large-scale sports sponsorship budget and a genuine, surprising F1 gap.</t>
+        </is>
+      </c>
+      <c r="O6" s="7" t="inlineStr">
+        <is>
+          <t>Lead with the Aflac Duck as a highly shareable, family-friendly F1 activation mascot/paddock character, paired with the Japan angle (Suzuka GP) given Aflac's outsized Japan business.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Orix Corporation</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>Public (TSE/NYSE), widely-held institutional shareholder base; no state or family control found</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Diversified financial services - leasing, corporate/PE investment, real estate, life insurance, renewable energy financing, aircraft/aviation leasing (global) - to corporates and retail investors across Japan, Asia, US and Europe</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>25k-50k (~35,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>TTM revenue ~$14.3B USD as of Sept 2026 (stockanalysis.com/companiesmarketcap); FY2025 net income record on base-profit growth - well above input's $18B estimate on the revenue line, corrected down but confirmed profitable and growing</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Market cap ~$43.3B USD as of June 3, 2026 (stockanalysis.com) - materially higher than input's ~$25B estimate; verified current</t>
+        </is>
+      </c>
+      <c r="K7" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Sells in 3+ markets (Japan, broader Asia, US/Europe aviation &amp; asset leasing) - pass; buyers span affluent retail (life insurance, wealth) and corporate decision-makers - pass; diversified industrial/financial conglomerate gives a workable precision-and-global-reach story - partial; category open - no diversified Japanese financial conglomerate on the F1 grid, and Japan hosts Suzuka GP giving a hometown hook. Customer scale mass-market + institutional (pass, note). No existing motorsport sponsorship found (owns NPB's Orix Buffaloes baseball club, new Under Armour teamwear deal 2026, but no F1/motorsport tie).</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>input's ~$25B market cap estimate was well stale/low - now ~$43B; use verified figure going forward</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>Mega-cap, profitable, growing, no existing F1/motorsport tie, and a strong Suzuka/Japan-GP hometown angle</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>Japan GP (Suzuka) hometown sponsor - pitch around precision engineering/asset performance (leasing, aviation, renewables) plus wealth/insurance storytelling for affluent Japanese and pan-Asian clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>CTBC Financial Holding</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>Public (TWSE); Koo family retains ~10-15% controlling influence via affiliates (Jeffrey Koo Jr. alone ~8.87%), foreign institutions ~43.5%; no state ownership found</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Banking, life insurance, securities to Taiwanese and regional (Asia) consumers/corporates</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>25k-50k (~28,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>TTM revenue ~US$8B equivalent (reported as S$10.63B, Aug 2026); H1 2026 net profit TWD39.5B, up 10% YoY - record high, shareholders' equity +59.5% YoY - clearly profitable and growing</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>Market cap ~TWD1.28T (~US$39B at ~32.5 TWD/USD) as of Aug 19, 2026 - substantially higher than input's ~$20B estimate; verified current (currency-converted, flag for finance team to confirm exact USD)</t>
+        </is>
+      </c>
+      <c r="K8" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>Sells Taiwan + regional Asia - partial market breadth; buyers include affluent life-insurance/wealth clients - pass; explicit 'global brand-building ambitions' (per input) plus proven large sports-marketing budget (first Taiwan company to own pro baseball, basketball AND esports teams, WBSC/World Baseball Classic sponsor) shows real capacity/appetite to spend - strong signal even though not yet a global-performance story; category open - no Taiwanese bank on the F1 grid. Mass-market + affluent customer scale (pass, note). No F1/motorsport tie found despite heavy sports-sponsorship history (baseball, basketball, golf, esports).</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>Taiwan HQ - note cross-strait/China-market optics if any messaging references mainland China</t>
+        </is>
+      </c>
+      <c r="N8" s="7" t="inlineStr">
+        <is>
+          <t>Mega-cap, record profits, no F1 tie, and an unusually active, well-funded sports-sponsorship track record signals real budget and appetite</t>
+        </is>
+      </c>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>Leverage CTBC's proven heavy sports-marketing spend (baseball/basketball/esports ownership) to pitch F1 as the next step up to a global platform for its international growth ambitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Hong Leong Bank</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>Malaysia</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>Public (Bursa Malaysia); Quek family-controlled via Hong Leong Financial Group - private, not state-linked</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Retail and commercial banking in Malaysia, Singapore, Vietnam and Cambodia</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>10k-25k (~10,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>FY2025 total income RM6.4B (~US$1.5B), +10.9% YoY, non-interest income +33.4% YoY - profitable and growing, matches input estimate</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Market cap ~$10.8B USD as of June 2026 (stockanalysis.com) - just above the $10B mega-brand threshold; verified current, up from input's ~$9B estimate</t>
+        </is>
+      </c>
+      <c r="K9" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>Sells across 4 ASEAN markets (Malaysia/Singapore/Vietnam/Cambodia) - pass; retail + growing non-interest/wealth income implies an affluent-leaning customer mix - partial pass; ASEAN-growth story is workable but not distinctly performance-tech; category wide open - regional retail banking is NOT taken on the F1 grid (Barclays/Santander/UBS are the taken global names) and no professional sports sponsorship found beyond internal staff events. Mass-market retail customer scale (pass, note).</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="inlineStr"/>
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t>Just cleared mega-brand threshold, profitable and growing, multi-market ASEAN reach, regional retail-banking category still open on the grid, no existing F1 tie</t>
+        </is>
+      </c>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>ASEAN growth/premier-banking story - use F1's expanding Southeast Asian fanbase to reach affluent, digitally engaged customers across Malaysia, Singapore, Vietnam and Cambodia</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Shriram Finance</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>Public (NSE/BSE); Shriram Group promoter entities plus private-equity investors (incl. TPG-linked holdings); no state ownership found</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Commercial vehicle, MSME and gold loans to Indian retail/SME customers, with strong rural/semi-urban reach</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>&gt;50k (~75,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Revenue growing strongly - Q2 revenue ₹10,090 Cr, +17.9% YoY; full-year figures point to roughly ₹48,000+ Cr (~US$5.5B), well above input's ~$3.5B estimate</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>Market cap ~₹242,034 Cr (~US$26.8B) as of Sept 15, 2026 - well above input's ~$13B estimate; verified current</t>
+        </is>
+      </c>
+      <c r="K10" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>Pan-India footprint across many states with distinct regional markets - reasonable market-breadth pass; SME/vehicle-owner buyers include real decision-makers even if not classic affluent urban 25-54; proven large sports-marketing budget (Pro Kabaddi League associate sponsor, cricket legend Rahul Dravid as brand ambassador, Padukone badminton school sponsorship) demonstrates real capacity/appetite - strong signal; category open - no Indian NBFC on the F1 grid. Mass-market/rural-semi-urban customer scale (pass, note). No F1/motorsport tie found.</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="inlineStr"/>
+      <c r="N10" s="7" t="inlineStr">
+        <is>
+          <t>Mega-cap, fast-growing NBFC with a proven, sizable sports-sponsorship budget (PKL, Dravid endorsement) and no existing F1 tie</t>
+        </is>
+      </c>
+      <c r="O10" s="7" t="inlineStr">
+        <is>
+          <t>Position F1 as the natural upgrade from Shriram's existing large-scale sports marketing (PKL, cricket icon endorsement) to a premium global platform, tapping India's rising affluent auto/finance customer base and any India GP revival buzz</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Cholamandalam Investment and Finance Company</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Chennai, India</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>Murugappa Group (Indian family-controlled industrial conglomerate) holds ~52% promoter stake; remainder publicly floated on NSE/BSE. No state, royal or sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Vehicle finance, home loans, and SME/loan-against-property lending across India</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>~40,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>$3.58B consolidated total income, FY2026 (ended Mar-2026: Rs 31,538.73 Cr, +20.6% YoY) - Screener/Whalesbook</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>~$17.9B market cap as of 4 Sep 2026 (Rs 1,57,063 Cr) - companiesmarketcap/valueresearchonline</t>
+        </is>
+      </c>
+      <c r="K11" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>Comfortably clears large-cap revenue/market-cap bar (market cap up ~28% vs prior Wave estimate). Profitable and growing fast (PAT +23% YoY to Rs 5,220 Cr, AUM +21% to Rs 2.43 lakh Cr) with no restructuring. Large retail customer base (vehicle/SME/home loan borrowers across India) gives real activation reach. No F1 or motorsport tie found for Cholamandalam or parent Murugappa Group.</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>NBFC sector remains subject to RBI regulatory tightening cycles; Figures are FY (Apr-Mar) based, ~6 months stale vs calendar Sept 2026</t>
+        </is>
+      </c>
+      <c r="N11" s="7" t="inlineStr">
+        <is>
+          <t>Large, profitable, fast-growing NBFC with strong capacity and no F1 conflicts or ownership blockers.</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>Position around India's growth-market motorsport fandom and vehicle-finance/auto-loan customer overlap with F1's expanding South Asian audience; tie to Murugappa Group's broader industrial/engineering ambitions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>L&amp;T Finance Holdings</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Mumbai, India</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>Majority-owned (~66%) by Larsen &amp; Toubro Limited, a professionally managed (non-family-promoter) Indian engineering conglomerate; free float on NSE/BSE. No state or sovereign control (state-owned LIC holds only a minor institutional stake, as with most large Indian listed cos).</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Rural/retail lending, two-wheeler and micro-loans, housing and infrastructure finance</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>~28,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>$2.04B total income, FY2026 (ended Mar-2026: Rs 17,917.03 Cr) - Kotak Neo/EquityBulls</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>~$8.8B market cap as of 11 Sep 2026 (Rs 77,471.36 Cr) - Tipranks/Stockanalysis</t>
+        </is>
+      </c>
+      <c r="K12" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>Market cap more than doubled vs prior Wave estimate ($4B est. -&gt; $8.8B actual) and clears the bar with room. Profitable and improving (FY26 PAT Rs 2,981 Cr, Q4 PAT Rs 806.63 Cr up YoY), post-transformation retail-lending strategy now stable, no active restructuring. Large rural/retail borrower base. No F1/motorsport tie found for L&amp;T Finance or parent Larsen &amp; Toubro.</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>Part of a diversified engineering parent (L&amp;T) that could itself be a separate, larger sponsorship prospect - avoid overlap/competing pitches</t>
+        </is>
+      </c>
+      <c r="N12" s="7" t="inlineStr">
+        <is>
+          <t>Solid, growing NBFC well above threshold with clean F1/ownership profile.</t>
+        </is>
+      </c>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>Engineering-pedigree brand story (L&amp;T Group heritage) paired with motorsport-technology narrative; rural/retail financial-inclusion growth story for activation reach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Poonawalla Fincorp</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>Pune, India</t>
+        </is>
+      </c>
+      <c r="F13" s="15" t="inlineStr">
+        <is>
+          <t>Cyrus Poonawalla Group (Adar Poonawalla / Serum Institute promoter family, majority private control) with public float on NSE/BSE. No state or sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Consumer and MSME lending, digital-first NBFC backed by the Poonawalla/Serum Institute family</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>~5,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>$772M total income, FY2026 (ended Mar-2026: Rs 6,795.65 Cr, +60% YoY) - Whalesbook/Screener</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>$4.34B market cap as of 4 Sep 2026 (Rs 42,215 Cr; +33% YoY) - stockanalysis</t>
+        </is>
+      </c>
+      <c r="K13" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>Market cap now clears $3B comfortably (up from the input's cautious ~$3.5B estimate) and revenue is smaller but growing 60% YoY. Capacity is 'improving' rather than steady-state: FY25 was a Rs 98 Cr net loss, and FY26 turned around to a Rs 541.8 Cr profit - a genuine swing, not a mature/stable earnings base. Checked specifically for Adar Poonawalla motorsport/F1 ties (he is a noted car collector) - found no existing Formula 1 or motorsport sponsorship by him or the group.</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>Recent (FY25) net loss before FY26 turnaround - capacity still stabilizing, not multi-year steady profitability; Smallest headcount/revenue base of this batch - verify org readiness for a sponsorship-scale program</t>
+        </is>
+      </c>
+      <c r="N13" s="7" t="inlineStr">
+        <is>
+          <t>Clears market-cap bar with strong momentum and no F1 conflict, though the profit turnaround is recent enough to note.</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>Promoter (Poonawalla family) already sports-sponsorship-active and a personal car/motorsport enthusiast - direct executive-level entry point; digital-first lending brand pairs well with F1's younger, digitally engaged fanbase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Grupo Aval Acciones y Valores</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Bogota, Colombia</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>Sarmiento Angulo family (Luis Carlos Sarmiento, majority private control) with free float on BVC/NYSE (ADR). No state or sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="inlineStr">
+        <is>
+          <t>Banking (Banco de Bogota, Banco de Occidente, AV Villas), pensions (Porvenir) across Colombia and Central America</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>~55,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <is>
+          <t>~$4.35B TTM revenue as of June 2026 (13.44 trillion COP LTM, +17.4% YoY) - stockanalysis/companiesmarketcap</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>~$5.5B market cap, ranged $5.0-6.0B through 2026 (latest ~$6.0B, Jan 2026 read) - stockanalysis/macrotrends</t>
+        </is>
+      </c>
+      <c r="K14" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>Clears the large-cap bar on both revenue and market cap, with double-digit revenue growth and a Q2 2026 earnings beat per its own transcript. Privately controlled, profitable, no restructuring signals. Colombia's largest financial group with genuine regional scale/customer base. Searched specifically for Sarmiento family/Grupo Aval motorsport ties - none found.</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="inlineStr">
+        <is>
+          <t>COP/USD conversion makes market cap figure sensitive to FX - reverify at time of outreach; Family-controlled with concentrated decision-making - identify the right entry point (Sarmiento family office vs. individual bank brands)</t>
+        </is>
+      </c>
+      <c r="N14" s="7" t="inlineStr">
+        <is>
+          <t>Dominant, profitable, privately-controlled regional financial group with no F1 conflicts.</t>
+        </is>
+      </c>
+      <c r="O14" s="7" t="inlineStr">
+        <is>
+          <t>Regional-champion narrative (largest financial group in Colombia, expanding into Central America) paired with F1's growing Latin American fan growth and the Mexico City/Miami GP footprint nearby.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Intercorp Financial Services</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>Lima, Peru</t>
+        </is>
+      </c>
+      <c r="F15" s="15" t="inlineStr">
+        <is>
+          <t>Controlled by the Rodriguez-Pastor family via Intercorp Peru Ltd. (majority private control); listed on NYSE and Lima exchange. No state or sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Banking (Interbank), insurance, and wealth management in Peru</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>~10,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>~$1.91B TTM revenue as of June 2026 - macrotrends/stockanalysis</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>~$6.4B market cap as of Sep 2026 (ranged $5.7-6.7B through the year) - stockanalysis/gurufocus</t>
+        </is>
+      </c>
+      <c r="K15" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>Market cap nearly double the Wave input's $3.5B estimate. Profitable and improving - management raised full-year ROE guidance above 17% on Q2 2026 earnings call, record net income in Q1 2026. Privately controlled diversified Peruvian financial group (Interbank consumer brand). Searched specifically for Interbank/Intercorp motorsport ties - none found.</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>Smaller headcount/geographic footprint (Peru-only) than some peers - confirm marketing budget scale for an F1-level sponsorship</t>
+        </is>
+      </c>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>Comfortably above threshold, improving profitability, no ownership or F1 blockers.</t>
+        </is>
+      </c>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>Interbank's strong retail/consumer brand recognition in Peru paired with F1's growth in Latin American viewership; family-office relationship entry point via Rodriguez-Pastor family.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Banco de Chile</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>Santiago, Chile</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>Controlled by the Luksic family (via Quinenco), with Citigroup holding a significant minority economic interest (~26%, non-controlling, via the LQIF joint venture structure) since a 2007 strategic alliance. No state or sovereign ownership; Citigroup stake is a minority flag, not a blocker.</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Retail and corporate banking in Chile</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>~13,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t>~$3.8B annualized run-rate, 2026 (Q2 2026 operating revenue CLP 922B, +20.9% YoY) - Investing.com/company results</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>$21.4B market cap as of 4 Sep 2026 (+44% YoY) - stockanalysis/companiesmarketcap</t>
+        </is>
+      </c>
+      <c r="K16" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t>Market cap well above (~65% higher than) the Wave input's $13B estimate and up 44% YoY - Chile's leading private bank with over a century of history. Q1 2026 net income dipped 18.3% YoY on higher provisioning, but Q2 2026 rebounded strongly (+20.9% revenue, ROE 27.9%) - overall improving, no restructuring. Searched specifically for Luksic family/Banco de Chile motorsport ties - none found. Citigroup's minority economic stake (non-controlling) confirmed as a strategic alliance, not a conflicting sponsorship agreement.</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t>Q1 2026 earnings dip on provisioning before Q2 rebound - monitor next quarter for trend confirmation; Citigroup minority stake (~26%) - unlikely to block a sponsorship decision but worth a light-touch conflict check given Citi's own global sponsorship portfolio</t>
+        </is>
+      </c>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t>Mega-cap, historic bank with strong recent momentum and no confirmed F1/motorsport conflicts.</t>
+        </is>
+      </c>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t>Century-plus heritage brand with Luksic family's broader international investment profile (Quinenco holds stakes across mining, beverages, shipping); position as a prestige, first-mover Chilean financial sponsor in F1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>Banco Davivienda</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>Bogota, Colombia</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>Controlled by Grupo Bolivar (Cortes family, majority private control); Scotiabank holds a ~20% minority stake since closing its Colombia/Costa Rica/Panama operations sale to Davivienda in Dec 2025. No state or sovereign ownership; Scotiabank stake is a minority flag.</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Retail/commercial banking across Colombia and Central America, now integrating former Scotiabank Colombia, Costa Rica and Panama operations under the 'DaviBank' brand</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>~17,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>~$2.8B annualized run-rate, 2026 est. (Q2 2026 revenue COP 2.84 trillion, +49% YoY on merger consolidation) - MarketScreener/Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>~$3.2B market cap as of Aug 2026 (COP 12.35 trillion) - Yahoo Finance</t>
+        </is>
+      </c>
+      <c r="K17" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>Market cap sits just above the $3B threshold as flagged in the input; the Scotiabank Colombia/Costa Rica/Panama merger (closed Dec 2025) is now integrated and driving strong results rather than dragging - Q2 2026 net income up ~50% YoY and revenue +49% YoY on consolidation, so capacity reads as improving, not distressed. Searched specifically for Grupo Bolivar/Sarmiento-adjacent Colombian banking motorsport ties - none found (note: Grupo Bolivar is Cortes-family controlled, distinct from the Sarmiento Angulo family behind Grupo Aval).</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>Market cap right at the large-cap threshold - reverify at outreach time given FX sensitivity (COP); Post-merger integration still maturing (DaviBank brand launched Dec 2025) - confirm marketing budget is not still constrained by integration costs; Scotiabank 20% minority stake - low-risk but worth a light conflict check given Scotiabank's own sponsorship activity</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t>Clears threshold with merger-driven growth momentum and no F1 conflicts, though scale and integration maturity warrant monitoring.</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>Newly-enlarged regional footprint (Colombia, Costa Rica, Panama) post-Scotiabank integration; DaviBank rebrand launch is a natural moment for a bold new marketing platform like F1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Storebrand</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Lysaker (Oslo area), Norway</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>Publicly listed on Oslo Bors, widely held, no state or founder-majority stake</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>Life insurance, pensions and sustainable asset management in Norway and Sweden</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>~2,300 (est.)</t>
+        </is>
+      </c>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>NOK 14.6B FY2025 (~$1.4B) (source: mynewsdesk.com Q4 2025 update / Storebrand IR)</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>~$8B market cap as of July 2026 (source: stockanalysis.com/companiesmarketcap.com)</t>
+        </is>
+      </c>
+      <c r="K18" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L18" s="7" t="inlineStr">
+        <is>
+          <t>Profitable, growing Nordic insurer/asset manager (record Q2 2026 results per earnings call); no state ownership; no F1 conflict identified.</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>ESG-forward brand identity would require a sustainability-framed pitch (F1 hybrid-power/net-zero-2030 angle) rather than a generic motorsport pitch</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr">
+        <is>
+          <t>Clean ownership, improving financial trajectory (record Q2 2026 results), and no competing F1 exposure.</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>Lead with F1's sustainability/hybrid-powertrain and net-zero-2030 narrative to match Storebrand's ESG-first brand positioning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Jyske Bank</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>Silkeborg, Denmark</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>Publicly listed, no state or single controlling shareholder</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Retail and private banking in Denmark</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>~3,800 (verified; sources show 3,803-3,851)</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>~€1.95B FY2024 (flat vs FY2023); FY2025 EPS +7% to DKK 85 (source: GlobeNewswire annual report Feb 2026)</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>~$9.19B market cap as of Aug 2026 (source: stockanalysis.com)</t>
+        </is>
+      </c>
+      <c r="K19" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>Denmark's third-largest bank, profitable with a record dividend (DKK 25/share) and a large new buyback (DKK 3.0B) announced off FY2025 results - clear capacity signal, no restructuring, no state ownership, no F1 conflict.</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>Some figures are estimates pending full FY2025 revenue confirmation in EUR terms</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>Profitable, capital-return-heavy bank with clean ownership and no F1 exposure to clear.</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>Position F1 hospitality/branding as a private-banking client acquisition and retention tool, leveraging the bank's record dividend/buyback momentum as a 'strength' narrative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>St. James's Place</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>Cirencester, United Kingdom</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>Publicly listed (LSE: STJ), widely held institutional ownership, no state stake</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>Wealth management and financial advice to UK affluent/retail clients</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>~4,500 (est.)</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>£30.2B FY2025 gross IFRS revenue (includes volatile policyholder investment return - not directly comparable to fee income) (source: stockanalysis.com); FUM record £220.0B FY2025, £240.8B H1 2026</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>£5.77B market cap as of Sept 2026 (source: companiesmarketcap.com)</t>
+        </is>
+      </c>
+      <c r="K20" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>UK's largest wealth manager; IFRS profit up 33% in 2025 and record FUM through H1 2026 show a clear post-restructuring recovery - the 2023 fee-charge controversy that prompted the rebuild is resolved, not ongoing.</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="inlineStr">
+        <is>
+          <t>Market cap (£5.77B) still below pre-2023 controversy peak - sentiment recovering but not fully restored; Reported £30.2B 'revenue' figure is IFRS gross including investment return, not core fee income - use with caution/footnote if citing externally</t>
+        </is>
+      </c>
+      <c r="N20" s="7" t="inlineStr">
+        <is>
+          <t>Clear, well-documented improving trajectory (record FUM, +33% profit) since the 2023 restructuring concluded; premium client base fits F1 hospitality well.</t>
+        </is>
+      </c>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>Premium UK wealth-management client base overlaps directly with F1 hospitality audiences; lean into the 'record FUM, comeback story' narrative for brand confidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>First Citizens BancShares</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Raleigh, NC, USA</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: FCNCA); Holding family retains significant voting control via Class B shares — no state/sovereign stake</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Commercial and retail banking (incl. former SVB assets) to US businesses and consumers</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>15,000–20,000</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>$9.03B FY2025 (down 3.2% YoY on lower SVB-loan accretion); net income ~$2.15–2.3B, per FY2025 results (SEC/stockanalysis.com)</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>~$24.3B market cap as of mid-Sept 2026 (stockanalysis.com)</t>
+        </is>
+      </c>
+      <c r="K21" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>Credit-cycle check: sector-wide regional-bank NPLs are declining and First Citizens' metrics track that trend; SVB venture-book concentration is a watch item but not distress — this is ongoing accretive integration, not restructuring. Large national commercial/retail bank (~$220B+ assets) with a strong tech/venture-capital client base via SVB. No F1 exposure. No sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>Revenue/net income declined YoY due to purchase-accounting accretion runoff on the SVB book — confirm this is a modeled glide path, not a credit problem, before pitching; Family-controlled voting structure (not a governance blocker, just note for stakeholder mapping)</t>
+        </is>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>Profitable, credit metrics healthy/improving, large scale, and a genuine tech/venture-client tie-in that could work well with F1's tech/innovation storyline.</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>Use the SVB/tech-and-innovation client base as the hook — a fintech/innovation-adjacent banking partner story rather than a generic regional-bank pitch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Regions Financial Corporation</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Birmingham, AL, USA</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>Public (NYSE: RF); widely held, no controlling shareholder</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Retail and commercial banking in the US Southeast/Midwest</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>15,000–20,000</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t>~$7.7B FY2025 total revenue (net interest + noninterest income; some aggregators show figures from $6.19B to $9.6B depending on methodology — use company 10-K for exact figure), record wealth/treasury-management income cited in FY2025 results</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>~$24.3B market cap as of early Sept 2026 (Forbes)</t>
+        </is>
+      </c>
+      <c r="K22" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t>Credit-cycle check: asset quality improving — NPL ratio down 4bps to 0.67%, criticized loans down 21% YoY, net charge-offs improving; consumer and commercial credit both described as healthy/stable. No restructuring. Large regional bank (~$155B assets) with broad Southeast/Midwest branch footprint. No F1 exposure; existing NFL/college-sports sponsor shows real sports-marketing budget and appetite.</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t>Revenue figure varies materially by data source — verify exact FY2025 total revenue against the 10-K before quoting in outreach</t>
+        </is>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
+        <is>
+          <t>Credit quality is genuinely improving (not just stable), the bank is profitable with record wealth-management income, and its existing regional sports-sponsorship culture (NFL, college sports) signals real appetite for a marquee marketing platform like F1.</t>
+        </is>
+      </c>
+      <c r="O22" s="7" t="inlineStr">
+        <is>
+          <t>Regional-growth and Southeast-expansion story — frame F1 US races (Miami, Austin, Las Vegas) as a natural extension of its existing regional sports-sponsorship playbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>Equitable Holdings, Inc.</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>New York, NY, USA</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>Public (NYSE: EQH); AXA S.A. fully divested its stake in 2021 (down to 0.07%, since sold) — no majority/foreign/sovereign owner today</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Life insurance, retirement/annuities, and asset management (majority owner of AllianceBernstein) for US consumers and institutions</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>10,000–15,000</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>~$14–15B FY2025 (est. — LTM revenue was $13.96B as of mid-2025, up 21% YoY; Q4 2025 revenue alone was $3.28B), per FY2025 results release</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>~$14.7B market cap as of mid-Sept 2026 (multiple sources)</t>
+        </is>
+      </c>
+      <c r="K23" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>Profitable, growing revenue, no restructuring. Large US insurer/asset-manager combo with a broad institutional and retail base. Ownership history flagged in input as AXA-linked is now moot — AXA fully exited in 2021, and Equitable has been building an independent brand identity since its 2020 rebrand from AXA Equitable. No F1 exposure. Not to be confused with EQB/Equitable Bank of Canada (different company).</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>Confirm full-year 2025 consolidated revenue figure directly from the 10-K — public aggregators give inconsistent line-item totals; Brand name overlap with Canada's EQB Equitable Bank — clarify identity in any outreach</t>
+        </is>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>Clean, fully independent public ownership (no residual AXA control despite the historical name), solid financial profile, and a rebuilding-brand-identity narrative that a marquee sponsorship like F1 could meaningfully accelerate.</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>Frame around the post-AXA independent-brand-building story — F1 as a platform to build Equitable's standalone identity distinct from its former AXA Equitable name, targeting HNW/retirement-planning audiences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>Primerica, Inc.</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>Duluth, GA, USA</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>Public (NYSE: PRI); widely held, no controlling shareholder</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Term life insurance and financial products distributed via ~130,000 independent licensed representatives to US/Canadian middle-income households</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>~3,000 employees plus ~130,000 independent licensed representatives</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="inlineStr">
+        <is>
+          <t>$3.29B FY2025 (up 6.6% YoY), per Q4/FY2025 results</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>~$9.0B market cap as of Sept 2026 (multiple sources, $8.85–9.07B range through 2026)</t>
+        </is>
+      </c>
+      <c r="K24" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
+          <t>Profitable, steady mid-single-digit growth, no restructuring. Very broad middle-income US/Canada consumer reach via its independent-rep distribution model — a large, dispersed audience base. No sponsor conflict found: no Primerica presence in current 2025/2026 NASCAR sponsor listings, though the company has a documented history of racing/motorsport-friendly marketing culture, which de-risks the 'will they even consider racing' question. No sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="M24" s="7" t="inlineStr">
+        <is>
+          <t>Confirm no dormant/legacy NASCAR contractual exclusivity remains before finalizing outreach, even though no active 2025/2026 NASCAR sponsorship was found</t>
+        </is>
+      </c>
+      <c r="N24" s="7" t="inlineStr">
+        <is>
+          <t>Financially solid, broad middle-market reach, and a demonstrated appetite for motorsport marketing with no current conflicting deal — a clean, plausible F1 prospect.</t>
+        </is>
+      </c>
+      <c r="O24" s="7" t="inlineStr">
+        <is>
+          <t>Use the massive independent-rep sales-force network as an activation and hospitality audience, and lean into the 'financial security for middle-income families' message alongside F1's broadening, family-oriented fanbase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Svenska Handelsbanken</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Stockholm, Sweden</t>
+        </is>
+      </c>
+      <c r="F25" s="17" t="inlineStr">
+        <is>
+          <t>Publicly listed; Oktogonen employee profit-sharing foundation holds ~8.2% of capital / 8.0% of votes (minority, not controlling)</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Retail and corporate banking across Sweden, UK, Netherlands and the Nordics</t>
+        </is>
+      </c>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>~12,200 (verified, FY2024 group headcount)</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>SEK 57.1B FY2025, down 9.3% YoY (source: MacroTrends/companiesmarketcap.com, 2026)</t>
+        </is>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>£22.83B market cap as of Aug 2026 (~$29B) (source: companiesmarketcap.com)</t>
+        </is>
+      </c>
+      <c r="K25" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L25" s="10" t="inlineStr">
+        <is>
+          <t>Major, profitable Nordic bank; no state or majority ownership issue (Oktogonen stake is minority/employee-linked); no F1 sponsorship conflict found. Revenue declined YoY in 2025 though earnings/ROE trends and UK/Netherlands lending growth remain positive.</t>
+        </is>
+      </c>
+      <c r="M25" s="10" t="inlineStr">
+        <is>
+          <t>Revenue down 9.3% YoY FY2025 - confirm cause (rate cycle) before pitching growth narrative; Historically conservative, low-key marketing culture (per input note) - gauge appetite before outreach</t>
+        </is>
+      </c>
+      <c r="N25" s="10" t="inlineStr">
+        <is>
+          <t>Meets financial/ownership bar but the bank's low-key marketing culture and a YoY revenue decline argue for a softer, relationship-led approach rather than a straight pitch.</t>
+        </is>
+      </c>
+      <c r="O25" s="10" t="inlineStr">
+        <is>
+          <t>Frame around Handelsbanken's UK/Netherlands growth push (offsetting flat Swedish home market) with a Silverstone/Zandvoort-linked relationship pitch rather than a mass-brand campaign.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>Sumitomo Mitsui Trust Holdings</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
+        <is>
+          <t>Public (TSE), separately listed from Sumitomo Mitsui Financial Group (SMFG) - confirmed distinct entity, not a duplicate; no state ownership found</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>Trust banking, asset management, real estate services to institutional and retail clients in Japan, with an asset-management arm serving global institutional clients</t>
+        </is>
+      </c>
+      <c r="H26" s="17" t="inlineStr">
+        <is>
+          <t>10k-25k (~20,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>Exact FY2025 revenue line not confirmed this pass; FY2025 net income forecast raised to ~JPY317B on gains from reducing strategic shareholdings, dividend raised - profitable and improving. Input's ~$9B FY2024 revenue estimate stands unverified (est.)</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t>Market cap ~$25.3B USD as of June 2026 (companiesmarketcap.com) - up from input's ~$18B estimate; verified current</t>
+        </is>
+      </c>
+      <c r="K26" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L26" s="10" t="inlineStr">
+        <is>
+          <t>Sells mostly domestic Japan with a global institutional asset-mgmt sleeve - partial market breadth (not clearly 3+ consumer markets); buyers are HNW/institutional and affluent trust clients - pass; story is wealth stewardship/trust rather than performance-tech-precision - weak fit; category open (no Japanese trust bank on F1 grid). Mass-affluent/institutional customer scale (pass, note). No motorsport sponsorship found.</t>
+        </is>
+      </c>
+      <c r="M26" s="10" t="inlineStr">
+        <is>
+          <t>revenue figure is an estimate this pass - not independently confirmed</t>
+        </is>
+      </c>
+      <c r="N26" s="10" t="inlineStr">
+        <is>
+          <t>Mega-cap and profitable with no F1 tie, but a narrower, Japan-centric trust/wealth franchise makes the growth/performance story harder to sell than a consumer-facing bank</t>
+        </is>
+      </c>
+      <c r="O26" s="10" t="inlineStr">
+        <is>
+          <t>Wealth-management/trust brand storytelling for HNW and institutional clients - legacy, precision and long-term stewardship themes tied to the Japan GP</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>TMBThanachart Bank (ttb)</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>Public (SET); Thai Ministry of Finance holds ~11.7% (largest legacy shareholder from FIDF/TMB recapitalization history) - MINORITY sovereign stake, flagged; Thanachart Capital and ING Groep also historic shareholders</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Retail/commercial banking and auto loans in Thailand</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="inlineStr">
+        <is>
+          <t>10k-25k (~14,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>TTM revenue ~$2.25B USD (Aug 2026); FY2025 revenue ~THB49.2B, roughly flat YoY (-0.72%) - profitable but not growing much, no active restructuring found</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>Market cap ~THB231B (~US$6.6B at ~35 THB/USD) as of July 2026 - above input's ~$4B estimate; verified current (currency-converted)</t>
+        </is>
+      </c>
+      <c r="K27" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L27" s="10" t="inlineStr">
+        <is>
+          <t>Single-market Thailand-only bank - fails 3+ market test; mass retail + auto-loan buyers, not distinctly affluent; plain retail-bank story; category open (no Thai bank on the F1 grid) - partial pass. Mass-market customer scale (pass, note).</t>
+        </is>
+      </c>
+      <c r="M27" s="10" t="inlineStr">
+        <is>
+          <t>Minority Thai Ministry of Finance stake (~11.7%) - state-linkage flag, not disqualifying</t>
+        </is>
+      </c>
+      <c r="N27" s="10" t="inlineStr">
+        <is>
+          <t>Meets the financial bar and no F1 tie, but single-market scale, flat growth and a minority state stake make the case thinner than regional peers like Hong Leong</t>
+        </is>
+      </c>
+      <c r="O27" s="10" t="inlineStr">
+        <is>
+          <t>If pursued, a narrow Thailand-only auto-finance/retail-banking angle; low priority without a stronger affluent or multi-market story</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>Yes Bank</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F28" s="17" t="inlineStr">
+        <is>
+          <t>Public (NSE/BSE); SMBC (Sumitomo Mitsui Banking Corp) now largest shareholder at ~24.9% (RBI-approved, deal completed Sept 2025); State Bank of India (SBI, majority Indian-government-owned) retains ~10.8% - MINORITY indirect sovereign linkage via SBI, flagged</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Retail and corporate banking in India</t>
+        </is>
+      </c>
+      <c r="H28" s="17" t="inlineStr">
+        <is>
+          <t>25k-50k (~25,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>Revenue ~₹30,658 Cr (~US$3.5B at ~88 INR/USD) - roughly matches input's ~$3B estimate</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>Market cap ~₹706.2B (~US$8.0B at ~88 INR/USD) as of Sept 2026 - within input's $7-8B range; verified current (currency-converted)</t>
+        </is>
+      </c>
+      <c r="K28" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L28" s="10" t="inlineStr">
+        <is>
+          <t>Single-market India-only bank - fails 3+ market test; mass retail buyers, not distinctly affluent; turnaround/credibility narrative (SMBC-backed, deposits returning per Japan Times) is a workable but not classic performance-tech story; category open (no Indian private bank on the F1 grid) - partial pass. Mass-market customer scale (pass, note). No F1/motorsport sponsorship found.</t>
+        </is>
+      </c>
+      <c r="M28" s="10" t="inlineStr">
+        <is>
+          <t>Ownership in transition - SMBC's 24.9% stake and new board influence per input; confirm current marketing/sponsorship decision authority before outreach; Minority indirect government linkage via SBI's ~10.8% stake</t>
+        </is>
+      </c>
+      <c r="N28" s="10" t="inlineStr">
+        <is>
+          <t>Improving turnaround with a credible new anchor investor (SMBC) and no F1 tie, but still a domestic-only mass-market bank with an ownership structure that needs confirming before outreach</t>
+        </is>
+      </c>
+      <c r="O28" s="10" t="inlineStr">
+        <is>
+          <t>"New chapter" turnaround/credibility story anchored by the SMBC partnership - confirm governance/marketing authority first, then pitch as India's re-emerging challenger bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>IIFL Finance</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Mumbai, India</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>Founder/promoter-led (Nirmal Jain and family, ~25% stake) with broad public float on NSE/BSE. No state or sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>Gold loans, housing finance, MSME/digital lending</t>
+        </is>
+      </c>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t>~30,000 (est.)</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>$1.52B consolidated total income, FY2026 (ended Mar-2026: Rs 13,373.83 Cr, +30.6% YoY) - Investing.com/Whalesbook</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>~$2.9B market cap as of 18 Sep 2026 (Rs 25,620.61 Cr) - stockanalysis/tickertape</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L29" s="10" t="inlineStr">
+        <is>
+          <t>Market cap has slipped below the $3B large-cap line (now SEBI-classified small-cap) despite the input flag calling it 'near threshold.' Fundamentals are recovering strongly - standalone business swung back to profit (Rs 1,153.5 Cr after an FY25 loss) and consolidated PAT up 214% YoY - but this reflects a bounce-back from the 2024 RBI gold-loan business restriction, not steady-state large-cap standing. Regulatory standing on gold loans is now resolved (new RBI tiered-LTV framework effective Apr-2026 applies industry-wide, not an IIFL-specific restriction). No F1/motorsport tie found.</t>
+        </is>
+      </c>
+      <c r="M29" s="10" t="inlineStr">
+        <is>
+          <t>Market cap currently below $3B large-cap threshold - re-verify at outreach time; 2024 RBI gold-loan restriction resolved but recency + still-recovering standalone profitability warrants monitoring</t>
+        </is>
+      </c>
+      <c r="N29" s="10" t="inlineStr">
+        <is>
+          <t>Recovering fast and no F1 conflict, but market cap has actually fallen below the large-cap bar this wave rather than just being 'near' it.</t>
+        </is>
+      </c>
+      <c r="O29" s="10" t="inlineStr">
+        <is>
+          <t>If pursued, frame around the digital-lending growth turnaround story and gold-loan-network customer scale; best revisited once market cap re-clears $3B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>3i Group</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>London, United Kingdom</t>
+        </is>
+      </c>
+      <c r="F30" s="17" t="inlineStr">
+        <is>
+          <t>Publicly listed investment trust (LSE: III), no state ownership</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>Private equity and infrastructure investment; NAV now ~77% concentrated in its Action retail stake (65.4%)</t>
+        </is>
+      </c>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t>~280-300 (verified small corporate/investment team; excludes Action's own ~250,000+ retail staff)</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>Not applicable - investment-return based; NAV £30.9B as of 31 Mar 2026, up 26% YoY (source: 3i.com FY26 press release)</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>~£23.8B market cap as of 29 Mar 2026 (~$30B) (source: massivemoats.substack.com)</t>
+        </is>
+      </c>
+      <c r="K30" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L30" s="10" t="inlineStr">
+        <is>
+          <t>Mega-cap by market value and NAV growth, fully profitable, no restructuring or ownership issue - but it is a ~280-person holding vehicle with no retail customer base of its own; 77% of value sits in one portfolio company (Action), which is the actual consumer-facing brand.</t>
+        </is>
+      </c>
+      <c r="M30" s="10" t="inlineStr">
+        <is>
+          <t>Extremely thin headcount/organization relative to market cap - typical for an investment trust but means no in-house marketing function to run a sponsorship; NAV heavily concentrated (77%) in a single asset (Action)</t>
+        </is>
+      </c>
+      <c r="N30" s="10" t="inlineStr">
+        <is>
+          <t>Financially exceeds the bar, but as a near-pure holding company it lacks the consumer/customer base and marketing organization that make an F1 partnership self-evidently useful; case rests on HNW investor relations, not product marketing.</t>
+        </is>
+      </c>
+      <c r="O30" s="10" t="inlineStr">
+        <is>
+          <t>Position as an HNW-investor/LP-facing prestige association (paddock club, investor days) rather than a mass-market brand sponsorship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>Intermediate Capital Group (ICG)</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>London, United Kingdom</t>
+        </is>
+      </c>
+      <c r="F31" s="17" t="inlineStr">
+        <is>
+          <t>Publicly listed (LSE: ICG), widely held, no state or controlling shareholder</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>Private credit and alternative asset management to institutional investors (pension funds, insurers, sovereign wealth funds)</t>
+        </is>
+      </c>
+      <c r="H31" s="17" t="inlineStr">
+        <is>
+          <t>~700-900 (est.)</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>£1,036M FY2026 total revenue; management fees £604M FY2025 (+19% YoY), fee-related earnings £350M FY2026 (+23% YoY) (source: icgam.com FY25 RNS / company reports)</t>
+        </is>
+      </c>
+      <c r="J31" s="10" t="inlineStr">
+        <is>
+          <t>~£5.4-6.7B market cap (2026, sources vary by date/currency) (source: companiesmarketcap.com)</t>
+        </is>
+      </c>
+      <c r="K31" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L31" s="10" t="inlineStr">
+        <is>
+          <t>Fast-growing, profitable UK alternative asset manager (AUM $126B) with no ownership/state issue and no restructuring - but its client base is exclusively institutional (LPs), with no retail/consumer customer to reach through F1.</t>
+        </is>
+      </c>
+      <c r="M31" s="10" t="inlineStr">
+        <is>
+          <t>Purely institutional (B2B) client base - limited 'customer scale' rationale for consumer-facing sponsorship; Confirmed distinct from unrelated 'Capital Group' entity per input flag - no naming conflict</t>
+        </is>
+      </c>
+      <c r="N31" s="10" t="inlineStr">
+        <is>
+          <t>Strong growth and profitability clear the capacity bar, but the institutional-only client base means the sponsorship case rests on LP relations/talent branding rather than mass-market marketing economics.</t>
+        </is>
+      </c>
+      <c r="O31" s="10" t="inlineStr">
+        <is>
+          <t>Frame as an LP-relationship and dealmaker-recruiting tool (paddock hospitality for institutional investors and prospective hires) rather than a consumer sponsorship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>Federated Hermes, Inc.</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>Pittsburgh, PA, USA</t>
+        </is>
+      </c>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>Public (NYSE: FHI); Donahue family controls majority voting power via Class B shares (no state/sovereign stake)</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>Money-market and active asset management for institutional and retail clients</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="inlineStr">
+        <is>
+          <t>1,000–5,000</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>$1.80B FY2025 (up 10.3% YoY, driven by higher money-market/equity AUM), per FY2025 earnings release/10-K (SEC)</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t>$4.45B market cap as of 11 Sep 2026 (MacroTrends/stockanalysis.com)</t>
+        </is>
+      </c>
+      <c r="K32" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L32" s="10" t="inlineStr">
+        <is>
+          <t>Profitable, record $911.6B AUM at Q2'26, no restructuring — capacity is fine but scale is modest ($4.45B cap, $1.8B revenue) relative to global F1 sponsorship costs. Customer base is institutional/retail asset-management clients, not a mass consumer brand. No F1/motorsport exposure. Ownership is US family-controlled public company, no sovereign/state stake.</t>
+        </is>
+      </c>
+      <c r="M32" s="10" t="inlineStr">
+        <is>
+          <t>Name collision: exclusion-list 'Hermes' entries likely refer to LVMH's Hermès (luxury goods, unrelated) — verify before outreach to avoid confusion/perception risk given Hermès's high visibility in F1 paddock fashion culture; Small ad/sponsorship budget relative to typical F1-tier deal size</t>
+        </is>
+      </c>
+      <c r="N32" s="10" t="inlineStr">
+        <is>
+          <t>Real, profitable, ownership-clean target, but sub-scale for a marquee F1 deal and carries meaningful brand-confusion risk with the LVMH Hermès name in F1-adjacent fashion/luxury circles.</t>
+        </is>
+      </c>
+      <c r="O32" s="10" t="inlineStr">
+        <is>
+          <t>Position around stewardship/responsible-investing (Hermes EOS) narrative tied to F1's sustainability push — likely a smaller regional/team-level activation rather than a series-level deal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>meets parameters</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>SLM Corporation (Sallie Mae)</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>Newark, DE / Salt Lake City, UT, USA</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>Public (NASDAQ: SLM); widely held, no controlling shareholder</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Private student loans and consumer banking to US students and families</t>
+        </is>
+      </c>
+      <c r="H33" s="17" t="inlineStr">
+        <is>
+          <t>1,000–2,500</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>$1.98B FY2025 (up from $1.84B FY2024), per Q4/FY2025 earnings release</t>
+        </is>
+      </c>
+      <c r="J33" s="10" t="inlineStr">
+        <is>
+          <t>~$4.7–4.8B market cap as of 19 Sept 2026 (stockanalysis.com)</t>
+        </is>
+      </c>
+      <c r="K33" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L33" s="10" t="inlineStr">
+        <is>
+          <t>Credit-cycle check (flagged per protocol): Q2 2026 delinquencies ticked up to 3.7% (from 3.5%) and net charge-offs rose to $113M (from $94M); management attributes a meaningful chunk of the increase to a specific fraud/debt-resolution-provider pattern affecting ~6.4% of gross charge-offs, and has moved recovery operations in-house — a real but contained credit issue, not a broad-based deterioration. Still profitable. Strong tie to the college-age/youth demographic F1 is actively courting. No F1 exposure. No sovereign ownership.</t>
+        </is>
+      </c>
+      <c r="M33" s="10" t="inlineStr">
+        <is>
+          <t>Stock has been volatile on 'elevated charge-off' headlines in 2026 — confirm the credit issue is resolved/contained before pitching a large sponsorship commitment; Small market cap (~$4.8B) relative to typical global F1 sponsorship spend</t>
+        </is>
+      </c>
+      <c r="N33" s="10" t="inlineStr">
+        <is>
+          <t>Genuinely strong youth/college-age audience overlap with F1's fan-growth strategy, but modest scale and an active, still-being-remediated credit-quality issue argue for caution or a smaller/regional deal rather than a marquee one.</t>
+        </is>
+      </c>
+      <c r="O33" s="10" t="inlineStr">
+        <is>
+          <t>College-age/young-fan acquisition story — align with F1's youth-fan growth push and financial-literacy-for-students messaging, likely sized as a mid-tier partnership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>exceeds - mega-brand</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>Mega Financial Holding</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>Taiwan</t>
+        </is>
+      </c>
+      <c r="F34" s="17" t="inlineStr">
+        <is>
+          <t>Public (TWSE); Ministry of Finance, R.O.C. holds ~8.2% (2025) as largest single shareholder - MINORITY sovereign stake, flagged per state-linkage check (not majority, does not trigger automatic No)</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>Commercial banking, insurance, securities, largely Taiwan-focused with an export-finance corporate client base</t>
+        </is>
+      </c>
+      <c r="H34" s="17" t="inlineStr">
+        <is>
+          <t>10k-25k (~14,000 est., unverified this pass)</t>
+        </is>
+      </c>
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>TTM revenue ~TWD78.9B (~US$2.4B); TTM profit ~TWD36.4B - profitable, no restructuring signals found</t>
+        </is>
+      </c>
+      <c r="J34" s="10" t="inlineStr">
+        <is>
+          <t>Market cap ~TWD593B (~US$18.2B at ~32.5 TWD/USD) - above input's ~$13B estimate; verified current (currency-converted)</t>
+        </is>
+      </c>
+      <c r="K34" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L34" s="10" t="inlineStr">
+        <is>
+          <t>Sells mostly within Taiwan with export-finance corporate reach - weak market breadth (not a clear 3+ consumer-market story); buyers are corporate/export-finance clients rather than affluent 25-54 retail - weak; plain commercial-bank story, little performance-tech-precision narrative; category technically open but weak fit overall. Mass-market/corporate customer scale (pass, note).</t>
+        </is>
+      </c>
+      <c r="M34" s="10" t="inlineStr">
+        <is>
+          <t>Minority Taiwan Ministry of Finance stake (~8.2%) - largest single shareholder is the state; flag for sponsor-ready optics review, not disqualifying</t>
+        </is>
+      </c>
+      <c r="N34" s="10" t="inlineStr">
+        <is>
+          <t>Mega-cap tier means it can't be a hard No, but the fit narrative is weak (Taiwan-only, corporate/export client base, minority state ownership)</t>
+        </is>
+      </c>
+      <c r="O34" s="10" t="inlineStr">
+        <is>
+          <t>If pursued, frame around Taiwan trade/export-finance and logistics network ties rather than a consumer affluence story; otherwise low priority vs. peers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>